<commit_message>
updated FAD and LAD column names
</commit_message>
<xml_diff>
--- a/bivalveTemplate.xlsx
+++ b/bivalveTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nheim01/Documents/PaleoSizeDB/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nheim01/Library/CloudStorage/Dropbox/size templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2578E6C-8DD2-934A-97E0-72B3CDC5CAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2034BF2F-9A82-2C43-953D-E602E9BD9671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="25240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="25240" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Subclass</t>
   </si>
@@ -55,18 +55,6 @@
     <t>Described by</t>
   </si>
   <si>
-    <t>Genus Origination Period</t>
-  </si>
-  <si>
-    <t>Genus Origination Epoch</t>
-  </si>
-  <si>
-    <t>Genus Extinction Period</t>
-  </si>
-  <si>
-    <t>Genus Extinction Epoch</t>
-  </si>
-  <si>
     <t>Figure Number</t>
   </si>
   <si>
@@ -88,15 +76,15 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>Bivalve Template</t>
+  </si>
+  <si>
     <t>Enterer</t>
   </si>
   <si>
     <t>Authority Year</t>
   </si>
   <si>
-    <t>Genus Origination Stage</t>
-  </si>
-  <si>
     <t>Specimen Period</t>
   </si>
   <si>
@@ -106,9 +94,6 @@
     <t>Specimen Stage</t>
   </si>
   <si>
-    <t>Genus Extinction Stage</t>
-  </si>
-  <si>
     <t>Specimen Biozone</t>
   </si>
   <si>
@@ -173,6 +158,24 @@
   </si>
   <si>
     <t>rl_length_left_mm</t>
+  </si>
+  <si>
+    <t>Genus/Subgenus Origination Period</t>
+  </si>
+  <si>
+    <t>Genus/Subgenus Origination Epoch</t>
+  </si>
+  <si>
+    <t>Genus/Subgenus Origination Stage</t>
+  </si>
+  <si>
+    <t>Genus/Subgenus Extinction Period</t>
+  </si>
+  <si>
+    <t>Genus/Subgenus Extinction Epoch</t>
+  </si>
+  <si>
+    <t>Genus/Subgenus Extinction Stage</t>
   </si>
 </sst>
 </file>
@@ -287,7 +290,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -317,6 +320,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1478,7 +1484,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:JC2"/>
+  <dimension ref="A1:JC3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="11.1640625" style="1" customWidth="1"/>
@@ -1494,12 +1500,12 @@
     <col min="11" max="11" width="19.6640625" style="2" customWidth="1"/>
     <col min="12" max="12" width="18.6640625" style="2" customWidth="1"/>
     <col min="13" max="13" width="18.33203125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="30" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="29.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="36" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="34.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="42.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="42.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="41.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="41.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="41" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="40.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17.83203125" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="23.33203125" style="2" bestFit="1" customWidth="1"/>
@@ -1534,427 +1540,484 @@
     <col min="264" max="16384" width="8.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:263" s="9" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:263" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B1" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="10"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
+      <c r="AF1" s="10"/>
+      <c r="AG1" s="10"/>
+      <c r="AH1" s="10"/>
+      <c r="AI1" s="10"/>
+      <c r="AJ1" s="10"/>
+      <c r="AK1" s="10"/>
+      <c r="AL1" s="10"/>
+      <c r="AM1" s="10"/>
+      <c r="AN1" s="10"/>
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="10"/>
+      <c r="AR1" s="10"/>
+      <c r="AS1" s="10"/>
+      <c r="AT1" s="10"/>
+      <c r="AU1" s="10"/>
+      <c r="AV1" s="10"/>
+      <c r="AW1" s="10"/>
+      <c r="AX1" s="10"/>
+      <c r="AY1" s="10"/>
+    </row>
+    <row r="2" spans="1:263" s="9" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="AF2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="3" t="s">
+      <c r="AG2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="P1" s="3" t="s">
+      <c r="AH2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Q1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="U1" s="3" t="s">
+      <c r="AI2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AK2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AL2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AM2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AN2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AO2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="AQ2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AR2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AS2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AT2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AU2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AV2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AX2" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AY2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="W1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="Y1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="AH1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="AK1" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="AL1" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="AM1" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AN1" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AO1" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="AP1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="AQ1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="AR1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="AS1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="AT1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AU1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="AV1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW1" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AX1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="AY1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="AZ1" s="8"/>
-      <c r="BA1" s="8"/>
-      <c r="BB1" s="8"/>
-      <c r="BC1" s="8"/>
-      <c r="BD1" s="8"/>
-      <c r="BE1" s="8"/>
-      <c r="BF1" s="8"/>
-      <c r="BG1" s="8"/>
-      <c r="BH1" s="8"/>
-      <c r="BI1" s="8"/>
-      <c r="BJ1" s="8"/>
-      <c r="BK1" s="8"/>
-      <c r="BL1" s="8"/>
-      <c r="BM1" s="8"/>
-      <c r="BN1" s="8"/>
-      <c r="BO1" s="8"/>
-      <c r="BP1" s="8"/>
-      <c r="BQ1" s="8"/>
-      <c r="BR1" s="8"/>
-      <c r="BS1" s="8"/>
-      <c r="BT1" s="8"/>
-      <c r="BU1" s="8"/>
-      <c r="BV1" s="8"/>
-      <c r="BW1" s="8"/>
-      <c r="BX1" s="8"/>
-      <c r="BY1" s="8"/>
-      <c r="BZ1" s="8"/>
-      <c r="CA1" s="8"/>
-      <c r="CB1" s="8"/>
-      <c r="CC1" s="8"/>
-      <c r="CD1" s="8"/>
-      <c r="CE1" s="8"/>
-      <c r="CF1" s="8"/>
-      <c r="CG1" s="8"/>
-      <c r="CH1" s="8"/>
-      <c r="CI1" s="8"/>
-      <c r="CJ1" s="8"/>
-      <c r="CK1" s="8"/>
-      <c r="CL1" s="8"/>
-      <c r="CM1" s="8"/>
-      <c r="CN1" s="8"/>
-      <c r="CO1" s="8"/>
-      <c r="CP1" s="8"/>
-      <c r="CQ1" s="8"/>
-      <c r="CR1" s="8"/>
-      <c r="CS1" s="8"/>
-      <c r="CT1" s="8"/>
-      <c r="CU1" s="8"/>
-      <c r="CV1" s="8"/>
-      <c r="CW1" s="8"/>
-      <c r="CX1" s="8"/>
-      <c r="CY1" s="8"/>
-      <c r="CZ1" s="8"/>
-      <c r="DA1" s="8"/>
-      <c r="DB1" s="8"/>
-      <c r="DC1" s="8"/>
-      <c r="DD1" s="8"/>
-      <c r="DE1" s="8"/>
-      <c r="DF1" s="8"/>
-      <c r="DG1" s="8"/>
-      <c r="DH1" s="8"/>
-      <c r="DI1" s="8"/>
-      <c r="DJ1" s="8"/>
-      <c r="DK1" s="8"/>
-      <c r="DL1" s="8"/>
-      <c r="DM1" s="8"/>
-      <c r="DN1" s="8"/>
-      <c r="DO1" s="8"/>
-      <c r="DP1" s="8"/>
-      <c r="DQ1" s="8"/>
-      <c r="DR1" s="8"/>
-      <c r="DS1" s="8"/>
-      <c r="DT1" s="8"/>
-      <c r="DU1" s="8"/>
-      <c r="DV1" s="8"/>
-      <c r="DW1" s="8"/>
-      <c r="DX1" s="8"/>
-      <c r="DY1" s="8"/>
-      <c r="DZ1" s="8"/>
-      <c r="EA1" s="8"/>
-      <c r="EB1" s="8"/>
-      <c r="EC1" s="8"/>
-      <c r="ED1" s="8"/>
-      <c r="EE1" s="8"/>
-      <c r="EF1" s="8"/>
-      <c r="EG1" s="8"/>
-      <c r="EH1" s="8"/>
-      <c r="EI1" s="8"/>
-      <c r="EJ1" s="8"/>
-      <c r="EK1" s="8"/>
-      <c r="EL1" s="8"/>
-      <c r="EM1" s="8"/>
-      <c r="EN1" s="8"/>
-      <c r="EO1" s="8"/>
-      <c r="EP1" s="8"/>
-      <c r="EQ1" s="8"/>
-      <c r="ER1" s="8"/>
-      <c r="ES1" s="8"/>
-      <c r="ET1" s="8"/>
-      <c r="EU1" s="8"/>
-      <c r="EV1" s="8"/>
-      <c r="EW1" s="8"/>
-      <c r="EX1" s="8"/>
-      <c r="EY1" s="8"/>
-      <c r="EZ1" s="8"/>
-      <c r="FA1" s="8"/>
-      <c r="FB1" s="8"/>
-      <c r="FC1" s="8"/>
-      <c r="FD1" s="8"/>
-      <c r="FE1" s="8"/>
-      <c r="FF1" s="8"/>
-      <c r="FG1" s="8"/>
-      <c r="FH1" s="8"/>
-      <c r="FI1" s="8"/>
-      <c r="FJ1" s="8"/>
-      <c r="FK1" s="8"/>
-      <c r="FL1" s="8"/>
-      <c r="FM1" s="8"/>
-      <c r="FN1" s="8"/>
-      <c r="FO1" s="8"/>
-      <c r="FP1" s="8"/>
-      <c r="FQ1" s="8"/>
-      <c r="FR1" s="8"/>
-      <c r="FS1" s="8"/>
-      <c r="FT1" s="8"/>
-      <c r="FU1" s="8"/>
-      <c r="FV1" s="8"/>
-      <c r="FW1" s="8"/>
-      <c r="FX1" s="8"/>
-      <c r="FY1" s="8"/>
-      <c r="FZ1" s="8"/>
-      <c r="GA1" s="8"/>
-      <c r="GB1" s="8"/>
-      <c r="GC1" s="8"/>
-      <c r="GD1" s="8"/>
-      <c r="GE1" s="8"/>
-      <c r="GF1" s="8"/>
-      <c r="GG1" s="8"/>
-      <c r="GH1" s="8"/>
-      <c r="GI1" s="8"/>
-      <c r="GJ1" s="8"/>
-      <c r="GK1" s="8"/>
-      <c r="GL1" s="8"/>
-      <c r="GM1" s="8"/>
-      <c r="GN1" s="8"/>
-      <c r="GO1" s="8"/>
-      <c r="GP1" s="8"/>
-      <c r="GQ1" s="8"/>
-      <c r="GR1" s="8"/>
-      <c r="GS1" s="8"/>
-      <c r="GT1" s="8"/>
-      <c r="GU1" s="8"/>
-      <c r="GV1" s="8"/>
-      <c r="GW1" s="8"/>
-      <c r="GX1" s="8"/>
-      <c r="GY1" s="8"/>
-      <c r="GZ1" s="8"/>
-      <c r="HA1" s="8"/>
-      <c r="HB1" s="8"/>
-      <c r="HC1" s="8"/>
-      <c r="HD1" s="8"/>
-      <c r="HE1" s="8"/>
-      <c r="HF1" s="8"/>
-      <c r="HG1" s="8"/>
-      <c r="HH1" s="8"/>
-      <c r="HI1" s="8"/>
-      <c r="HJ1" s="8"/>
-      <c r="HK1" s="8"/>
-      <c r="HL1" s="8"/>
-      <c r="HM1" s="8"/>
-      <c r="HN1" s="8"/>
-      <c r="HO1" s="8"/>
-      <c r="HP1" s="8"/>
-      <c r="HQ1" s="8"/>
-      <c r="HR1" s="8"/>
-      <c r="HS1" s="8"/>
-      <c r="HT1" s="8"/>
-      <c r="HU1" s="8"/>
-      <c r="HV1" s="8"/>
-      <c r="HW1" s="8"/>
-      <c r="HX1" s="8"/>
-      <c r="HY1" s="8"/>
-      <c r="HZ1" s="8"/>
-      <c r="IA1" s="8"/>
-      <c r="IB1" s="8"/>
-      <c r="IC1" s="8"/>
-      <c r="ID1" s="8"/>
-      <c r="IE1" s="8"/>
-      <c r="IF1" s="8"/>
-      <c r="IG1" s="8"/>
-      <c r="IH1" s="8"/>
-      <c r="II1" s="8"/>
-      <c r="IJ1" s="8"/>
-      <c r="IK1" s="8"/>
-      <c r="IL1" s="8"/>
-      <c r="IM1" s="8"/>
-      <c r="IN1" s="8"/>
-      <c r="IO1" s="8"/>
-      <c r="IP1" s="8"/>
-      <c r="IQ1" s="8"/>
-      <c r="IR1" s="8"/>
-      <c r="IS1" s="8"/>
-      <c r="IT1" s="8"/>
-      <c r="IU1" s="8"/>
-      <c r="IV1" s="8"/>
-      <c r="IW1" s="8"/>
-      <c r="IX1" s="8"/>
-      <c r="IY1" s="8"/>
-      <c r="IZ1" s="8"/>
-      <c r="JA1" s="8"/>
-      <c r="JB1" s="8"/>
-      <c r="JC1" s="8"/>
+      <c r="AZ2" s="8"/>
+      <c r="BA2" s="8"/>
+      <c r="BB2" s="8"/>
+      <c r="BC2" s="8"/>
+      <c r="BD2" s="8"/>
+      <c r="BE2" s="8"/>
+      <c r="BF2" s="8"/>
+      <c r="BG2" s="8"/>
+      <c r="BH2" s="8"/>
+      <c r="BI2" s="8"/>
+      <c r="BJ2" s="8"/>
+      <c r="BK2" s="8"/>
+      <c r="BL2" s="8"/>
+      <c r="BM2" s="8"/>
+      <c r="BN2" s="8"/>
+      <c r="BO2" s="8"/>
+      <c r="BP2" s="8"/>
+      <c r="BQ2" s="8"/>
+      <c r="BR2" s="8"/>
+      <c r="BS2" s="8"/>
+      <c r="BT2" s="8"/>
+      <c r="BU2" s="8"/>
+      <c r="BV2" s="8"/>
+      <c r="BW2" s="8"/>
+      <c r="BX2" s="8"/>
+      <c r="BY2" s="8"/>
+      <c r="BZ2" s="8"/>
+      <c r="CA2" s="8"/>
+      <c r="CB2" s="8"/>
+      <c r="CC2" s="8"/>
+      <c r="CD2" s="8"/>
+      <c r="CE2" s="8"/>
+      <c r="CF2" s="8"/>
+      <c r="CG2" s="8"/>
+      <c r="CH2" s="8"/>
+      <c r="CI2" s="8"/>
+      <c r="CJ2" s="8"/>
+      <c r="CK2" s="8"/>
+      <c r="CL2" s="8"/>
+      <c r="CM2" s="8"/>
+      <c r="CN2" s="8"/>
+      <c r="CO2" s="8"/>
+      <c r="CP2" s="8"/>
+      <c r="CQ2" s="8"/>
+      <c r="CR2" s="8"/>
+      <c r="CS2" s="8"/>
+      <c r="CT2" s="8"/>
+      <c r="CU2" s="8"/>
+      <c r="CV2" s="8"/>
+      <c r="CW2" s="8"/>
+      <c r="CX2" s="8"/>
+      <c r="CY2" s="8"/>
+      <c r="CZ2" s="8"/>
+      <c r="DA2" s="8"/>
+      <c r="DB2" s="8"/>
+      <c r="DC2" s="8"/>
+      <c r="DD2" s="8"/>
+      <c r="DE2" s="8"/>
+      <c r="DF2" s="8"/>
+      <c r="DG2" s="8"/>
+      <c r="DH2" s="8"/>
+      <c r="DI2" s="8"/>
+      <c r="DJ2" s="8"/>
+      <c r="DK2" s="8"/>
+      <c r="DL2" s="8"/>
+      <c r="DM2" s="8"/>
+      <c r="DN2" s="8"/>
+      <c r="DO2" s="8"/>
+      <c r="DP2" s="8"/>
+      <c r="DQ2" s="8"/>
+      <c r="DR2" s="8"/>
+      <c r="DS2" s="8"/>
+      <c r="DT2" s="8"/>
+      <c r="DU2" s="8"/>
+      <c r="DV2" s="8"/>
+      <c r="DW2" s="8"/>
+      <c r="DX2" s="8"/>
+      <c r="DY2" s="8"/>
+      <c r="DZ2" s="8"/>
+      <c r="EA2" s="8"/>
+      <c r="EB2" s="8"/>
+      <c r="EC2" s="8"/>
+      <c r="ED2" s="8"/>
+      <c r="EE2" s="8"/>
+      <c r="EF2" s="8"/>
+      <c r="EG2" s="8"/>
+      <c r="EH2" s="8"/>
+      <c r="EI2" s="8"/>
+      <c r="EJ2" s="8"/>
+      <c r="EK2" s="8"/>
+      <c r="EL2" s="8"/>
+      <c r="EM2" s="8"/>
+      <c r="EN2" s="8"/>
+      <c r="EO2" s="8"/>
+      <c r="EP2" s="8"/>
+      <c r="EQ2" s="8"/>
+      <c r="ER2" s="8"/>
+      <c r="ES2" s="8"/>
+      <c r="ET2" s="8"/>
+      <c r="EU2" s="8"/>
+      <c r="EV2" s="8"/>
+      <c r="EW2" s="8"/>
+      <c r="EX2" s="8"/>
+      <c r="EY2" s="8"/>
+      <c r="EZ2" s="8"/>
+      <c r="FA2" s="8"/>
+      <c r="FB2" s="8"/>
+      <c r="FC2" s="8"/>
+      <c r="FD2" s="8"/>
+      <c r="FE2" s="8"/>
+      <c r="FF2" s="8"/>
+      <c r="FG2" s="8"/>
+      <c r="FH2" s="8"/>
+      <c r="FI2" s="8"/>
+      <c r="FJ2" s="8"/>
+      <c r="FK2" s="8"/>
+      <c r="FL2" s="8"/>
+      <c r="FM2" s="8"/>
+      <c r="FN2" s="8"/>
+      <c r="FO2" s="8"/>
+      <c r="FP2" s="8"/>
+      <c r="FQ2" s="8"/>
+      <c r="FR2" s="8"/>
+      <c r="FS2" s="8"/>
+      <c r="FT2" s="8"/>
+      <c r="FU2" s="8"/>
+      <c r="FV2" s="8"/>
+      <c r="FW2" s="8"/>
+      <c r="FX2" s="8"/>
+      <c r="FY2" s="8"/>
+      <c r="FZ2" s="8"/>
+      <c r="GA2" s="8"/>
+      <c r="GB2" s="8"/>
+      <c r="GC2" s="8"/>
+      <c r="GD2" s="8"/>
+      <c r="GE2" s="8"/>
+      <c r="GF2" s="8"/>
+      <c r="GG2" s="8"/>
+      <c r="GH2" s="8"/>
+      <c r="GI2" s="8"/>
+      <c r="GJ2" s="8"/>
+      <c r="GK2" s="8"/>
+      <c r="GL2" s="8"/>
+      <c r="GM2" s="8"/>
+      <c r="GN2" s="8"/>
+      <c r="GO2" s="8"/>
+      <c r="GP2" s="8"/>
+      <c r="GQ2" s="8"/>
+      <c r="GR2" s="8"/>
+      <c r="GS2" s="8"/>
+      <c r="GT2" s="8"/>
+      <c r="GU2" s="8"/>
+      <c r="GV2" s="8"/>
+      <c r="GW2" s="8"/>
+      <c r="GX2" s="8"/>
+      <c r="GY2" s="8"/>
+      <c r="GZ2" s="8"/>
+      <c r="HA2" s="8"/>
+      <c r="HB2" s="8"/>
+      <c r="HC2" s="8"/>
+      <c r="HD2" s="8"/>
+      <c r="HE2" s="8"/>
+      <c r="HF2" s="8"/>
+      <c r="HG2" s="8"/>
+      <c r="HH2" s="8"/>
+      <c r="HI2" s="8"/>
+      <c r="HJ2" s="8"/>
+      <c r="HK2" s="8"/>
+      <c r="HL2" s="8"/>
+      <c r="HM2" s="8"/>
+      <c r="HN2" s="8"/>
+      <c r="HO2" s="8"/>
+      <c r="HP2" s="8"/>
+      <c r="HQ2" s="8"/>
+      <c r="HR2" s="8"/>
+      <c r="HS2" s="8"/>
+      <c r="HT2" s="8"/>
+      <c r="HU2" s="8"/>
+      <c r="HV2" s="8"/>
+      <c r="HW2" s="8"/>
+      <c r="HX2" s="8"/>
+      <c r="HY2" s="8"/>
+      <c r="HZ2" s="8"/>
+      <c r="IA2" s="8"/>
+      <c r="IB2" s="8"/>
+      <c r="IC2" s="8"/>
+      <c r="ID2" s="8"/>
+      <c r="IE2" s="8"/>
+      <c r="IF2" s="8"/>
+      <c r="IG2" s="8"/>
+      <c r="IH2" s="8"/>
+      <c r="II2" s="8"/>
+      <c r="IJ2" s="8"/>
+      <c r="IK2" s="8"/>
+      <c r="IL2" s="8"/>
+      <c r="IM2" s="8"/>
+      <c r="IN2" s="8"/>
+      <c r="IO2" s="8"/>
+      <c r="IP2" s="8"/>
+      <c r="IQ2" s="8"/>
+      <c r="IR2" s="8"/>
+      <c r="IS2" s="8"/>
+      <c r="IT2" s="8"/>
+      <c r="IU2" s="8"/>
+      <c r="IV2" s="8"/>
+      <c r="IW2" s="8"/>
+      <c r="IX2" s="8"/>
+      <c r="IY2" s="8"/>
+      <c r="IZ2" s="8"/>
+      <c r="JA2" s="8"/>
+      <c r="JB2" s="8"/>
+      <c r="JC2" s="8"/>
     </row>
-    <row r="2" spans="1:263" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
-      <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
-      <c r="Y2" s="6"/>
-      <c r="Z2" s="6"/>
-      <c r="AA2" s="6"/>
-      <c r="AB2" s="6"/>
-      <c r="AC2" s="6"/>
-      <c r="AD2" s="6"/>
-      <c r="AE2" s="6"/>
-      <c r="AF2" s="6"/>
-      <c r="AG2" s="6"/>
-      <c r="AH2" s="6"/>
-      <c r="AI2" s="6"/>
-      <c r="AJ2" s="6"/>
-      <c r="AK2" s="6"/>
-      <c r="AL2" s="6"/>
-      <c r="AM2" s="6"/>
-      <c r="AN2" s="6"/>
-      <c r="AO2" s="6"/>
-      <c r="AP2" s="6"/>
-      <c r="AQ2" s="6"/>
-      <c r="AR2" s="6"/>
-      <c r="AS2" s="6"/>
-      <c r="AT2" s="6"/>
-      <c r="AU2" s="6"/>
-      <c r="AV2" s="6"/>
-      <c r="AW2" s="6"/>
-      <c r="AX2" s="6"/>
-      <c r="AY2" s="6"/>
+    <row r="3" spans="1:263" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="6"/>
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="6"/>
+      <c r="AJ3" s="6"/>
+      <c r="AK3" s="6"/>
+      <c r="AL3" s="6"/>
+      <c r="AM3" s="6"/>
+      <c r="AN3" s="6"/>
+      <c r="AO3" s="6"/>
+      <c r="AP3" s="6"/>
+      <c r="AQ3" s="6"/>
+      <c r="AR3" s="6"/>
+      <c r="AS3" s="6"/>
+      <c r="AT3" s="6"/>
+      <c r="AU3" s="6"/>
+      <c r="AV3" s="6"/>
+      <c r="AW3" s="6"/>
+      <c r="AX3" s="6"/>
+      <c r="AY3" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:AY1"/>
+  </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
   <headerFooter>

</xml_diff>